<commit_message>
chore: commit remaining assets, spreadsheet templates, and configurations
</commit_message>
<xml_diff>
--- a/backend/data/role_applications.xlsx
+++ b/backend/data/role_applications.xlsx
@@ -5,7 +5,7 @@
   <sheets>
     <sheet name="Contributors" sheetId="1" r:id="rId1"/>
     <sheet name="Ambassadors" sheetId="2" r:id="rId2"/>
-    <sheet name="Sponsors" sheetId="3" r:id="rId3"/>
+    <sheet name="Project Admins" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -399,16 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" customWidth="1"/>
-    <col min="4" max="4" width="27.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="37.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,255 +415,48 @@
         <v>Email</v>
       </c>
       <c r="E1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="F1" t="str">
         <v>GitHub</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Tech Stack</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Status</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>28/6/2026, 10:33:49 am</v>
+        <v>17/7/2026, 12:02:20 am</v>
       </c>
       <c r="B2" t="str">
         <v>Contributor</v>
       </c>
       <c r="C2" t="str">
-        <v>Test Contributor</v>
+        <v>Om</v>
       </c>
       <c r="D2" t="str">
-        <v>test_contrib@example.com</v>
+        <v>omparkhi1@gmail.com</v>
       </c>
       <c r="E2" t="str">
-        <v>testgithubuser</v>
+        <v>Pending</v>
       </c>
       <c r="F2" t="str">
-        <v>React, Node.js</v>
+        <v>github.com/om</v>
       </c>
       <c r="G2" t="str">
-        <v>Approved</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>28/6/2026, 10:36:03 am</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Om Vijay Parkhi</v>
-      </c>
-      <c r="D3" t="str">
-        <v>parkhiom50@gmail.com</v>
-      </c>
-      <c r="E3" t="str">
-        <v>https://github.com/omparkhi</v>
-      </c>
-      <c r="F3" t="str">
-        <v>MERN</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Approved</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>28/6/2026, 10:44:00 am</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Test Contributor</v>
-      </c>
-      <c r="D4" t="str">
-        <v>test_contrib@example.com</v>
-      </c>
-      <c r="E4" t="str">
-        <v>testgithubuser</v>
-      </c>
-      <c r="F4" t="str">
-        <v>React, Node.js</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Pending</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>28/6/2026, 10:45:06 am</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Test Contributor</v>
-      </c>
-      <c r="D5" t="str">
-        <v>test_contrib@example.com</v>
-      </c>
-      <c r="E5" t="str">
-        <v>testgithubuser</v>
-      </c>
-      <c r="F5" t="str">
-        <v>React, Node.js</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Pending</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>28/6/2026, 10:46:13 am</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Om Vijay Parkhi</v>
-      </c>
-      <c r="D6" t="str">
-        <v>parkhiom50@gmail.com</v>
-      </c>
-      <c r="E6" t="str">
-        <v>https://github.com/omparkhi</v>
-      </c>
-      <c r="F6" t="str">
-        <v>MERN</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Pending</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>28/6/2026, 10:51:42 am</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Test Contributor</v>
-      </c>
-      <c r="D7" t="str">
-        <v>test_contrib@example.com</v>
-      </c>
-      <c r="E7" t="str">
-        <v>testgithubuser</v>
-      </c>
-      <c r="F7" t="str">
-        <v>React, Node.js</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Pending</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>28/6/2026, 10:54:47 am</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Om</v>
-      </c>
-      <c r="D8" t="str">
-        <v>omparkhi23@gmail.com</v>
-      </c>
-      <c r="E8" t="str">
-        <v>https://github.com/omparkhi</v>
-      </c>
-      <c r="F8" t="str">
-        <v>React, Node, Express, Monhgodb, js</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Approved</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>28/6/2026, 11:09:27 am</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Test Contributor</v>
-      </c>
-      <c r="D9" t="str">
-        <v>test_contrib@example.com</v>
-      </c>
-      <c r="E9" t="str">
-        <v>testgithubuser</v>
-      </c>
-      <c r="F9" t="str">
-        <v>React, Node.js</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Pending</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>28/6/2026, 2:13:52 pm</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Om Vijay Parkhi</v>
-      </c>
-      <c r="D10" t="str">
-        <v>omparkhi23@gmail.com</v>
-      </c>
-      <c r="E10" t="str">
-        <v>https://github.com/omparkhi</v>
-      </c>
-      <c r="F10" t="str">
-        <v>React, Node, Express, MongoDB, JS</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Pending</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>2/7/2026, 11:14:13 pm</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Contributor</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Om</v>
-      </c>
-      <c r="D11" t="str">
-        <v>parkhiom5@gmail.com</v>
-      </c>
-      <c r="E11" t="str">
-        <v>https://github.com/omparkhi</v>
-      </c>
-      <c r="F11" t="str">
-        <v>React, Node, Express, MongoDB, JS</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Approved</v>
+        <v>mern</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -688,54 +472,71 @@
         <v>Email</v>
       </c>
       <c r="E1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="F1" t="str">
         <v>GitHub</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>College</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Year</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Motivation</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>28/6/2026, 10:33:52 am</v>
+        <v>17/7/2026, 12:02:57 am</v>
       </c>
       <c r="B2" t="str">
         <v>Ambassador</v>
       </c>
       <c r="C2" t="str">
-        <v>Test Contributor</v>
+        <v>Om</v>
       </c>
       <c r="D2" t="str">
-        <v>test_contrib@example.com</v>
+        <v>omparkhi1@gmail.com</v>
       </c>
       <c r="E2" t="str">
-        <v>testgithubuser</v>
+        <v>Pending</v>
       </c>
       <c r="F2" t="str">
-        <v>State Tech University</v>
+        <v>github.com/om</v>
       </c>
       <c r="G2" t="str">
-        <v>3rd Year</v>
+        <v>TARS</v>
       </c>
       <c r="H2" t="str">
-        <v>I love hosting student hackathons!</v>
+        <v>1st Year</v>
+      </c>
+      <c r="I2" t="str">
+        <v>kjfjjvj</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:I3"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="50.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -751,41 +552,82 @@
         <v>Email</v>
       </c>
       <c r="E1" t="str">
-        <v>Company</v>
+        <v>Status</v>
       </c>
       <c r="F1" t="str">
-        <v>Sponsorship Tier</v>
+        <v>GitHub</v>
       </c>
       <c r="G1" t="str">
-        <v>Message / Suggestions</v>
+        <v>Project Name</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Repository URL</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Motivation</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>28/6/2026, 10:33:55 am</v>
+        <v>17/7/2026, 12:58:06 am</v>
       </c>
       <c r="B2" t="str">
-        <v>Sponsor</v>
+        <v>Project Admin</v>
       </c>
       <c r="C2" t="str">
-        <v>Acme Corp Rep</v>
+        <v>Om</v>
       </c>
       <c r="D2" t="str">
-        <v>sponsor@acme.com</v>
+        <v>parkhiom5@gmail.com</v>
       </c>
       <c r="E2" t="str">
-        <v>Acme Corp</v>
+        <v>Pending</v>
       </c>
       <c r="F2" t="str">
-        <v>Gold Tier</v>
+        <v/>
       </c>
       <c r="G2" t="str">
-        <v>We'd love to fund hoodies and sandbox credits.</v>
+        <v xml:space="preserve">test, test2 </v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://github.com/RonitNagose, https://github.com/RonitNagose</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>17/7/2026, 1:02:49 am</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Project Admin</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Om</v>
+      </c>
+      <c r="D3" t="str">
+        <v>parkhiom5@gmail.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>test1, test</v>
+      </c>
+      <c r="H3" t="str">
+        <v xml:space="preserve"> https://github.com/RonitNagose,  https://github.com/RonitNagose</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: attach badges to approved emails and add backfill script
</commit_message>
<xml_diff>
--- a/backend/data/role_applications.xlsx
+++ b/backend/data/role_applications.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -447,9 +447,32 @@
         <v>mern</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>17/7/2026, 10:45:34 pm</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Contributor</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Om2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>parkhiom5@gmail.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://github.com/omparkhi</v>
+      </c>
+      <c r="G3" t="str">
+        <v>mern</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -525,12 +548,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
@@ -625,9 +648,67 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>17/7/2026, 10:59:09 pm</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Project Admin</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Ronit2</v>
+      </c>
+      <c r="D4" t="str">
+        <v>nagoseronit18@gmail.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>New Project</v>
+      </c>
+      <c r="H4" t="str">
+        <v>https://github.com/omparkhi/Simon-Say-Game</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>17/7/2026, 11:05:07 pm</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Project Admin</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Altraverse</v>
+      </c>
+      <c r="D5" t="str">
+        <v>altraverse5@gmail.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>Simon Game</v>
+      </c>
+      <c r="H5" t="str">
+        <v>https://github.com/omparkhi/Simon-Say-Game</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Add project edit and base64 image upload
</commit_message>
<xml_diff>
--- a/backend/data/role_applications.xlsx
+++ b/backend/data/role_applications.xlsx
@@ -399,7 +399,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I4"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="23.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,6 +432,12 @@
       <c r="G1" t="str">
         <v>Tech Stack</v>
       </c>
+      <c r="H1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="I1" t="str">
+        <v>LinkedIn</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -470,16 +485,45 @@
         <v>mern</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>23/7/2026, 5:35:37 pm</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Contributor</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Om Parkhi</v>
+      </c>
+      <c r="D4" t="str">
+        <v>parkhiom50@gmail.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Rejected</v>
+      </c>
+      <c r="F4" t="str">
+        <v>https://github.com/omparkhi</v>
+      </c>
+      <c r="G4" t="str">
+        <v>MERN</v>
+      </c>
+      <c r="H4" t="str">
+        <v>9657954641</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -539,27 +583,103 @@
         <v>kjfjjvj</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>18/7/2026, 12:22:23 am</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Ambassador</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Altraverse</v>
+      </c>
+      <c r="D3" t="str">
+        <v>altraverse5@gmail.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://github.com/omparkhi</v>
+      </c>
+      <c r="G3" t="str">
+        <v>PBCOE</v>
+      </c>
+      <c r="H3" t="str">
+        <v>4th Year</v>
+      </c>
+      <c r="I3" t="str">
+        <v>hii</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>19/7/2026, 11:46:59 pm</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Ambassador</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Om Parkhi</v>
+      </c>
+      <c r="D4" t="str">
+        <v>parkhiom50@gmail.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>PBCOE</v>
+      </c>
+      <c r="H4" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="I4" t="str">
+        <v>jhjjh</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>20/7/2026, 1:03:35 am</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Ambassador</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Yogesh</v>
+      </c>
+      <c r="D5" t="str">
+        <v>parkhiom5@gmail.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>TARS</v>
+      </c>
+      <c r="H5" t="str">
+        <v>1st Year</v>
+      </c>
+      <c r="I5" t="str">
+        <v>hii</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.83203125" customWidth="1"/>
-    <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="50.83203125" customWidth="1"/>
-    <col min="9" max="9" width="13.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:I6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -706,9 +826,38 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>20/7/2026, 1:08:16 am</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Project Admin</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Altraverse</v>
+      </c>
+      <c r="D6" t="str">
+        <v>altraverse5@gmail.com</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>Tars</v>
+      </c>
+      <c r="H6" t="str">
+        <v>https://github.com/om</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add project admin live status tracking, webhook sync, timeline, and banner assets
</commit_message>
<xml_diff>
--- a/backend/data/role_applications.xlsx
+++ b/backend/data/role_applications.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -453,7 +453,7 @@
         <v>omparkhi1@gmail.com</v>
       </c>
       <c r="E2" t="str">
-        <v>Pending</v>
+        <v>Approved</v>
       </c>
       <c r="F2" t="str">
         <v>github.com/om</v>
@@ -514,9 +514,38 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>22/8/2026, 1:07:07 am</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Contributor</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Om</v>
+      </c>
+      <c r="D5" t="str">
+        <v>omparkhi1@gmail.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="F5" t="str">
+        <v>https://github.com/om07-dev</v>
+      </c>
+      <c r="G5" t="str">
+        <v>MERN</v>
+      </c>
+      <c r="H5" t="str">
+        <v>9657954641</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>